<commit_message>
update CR + egine
</commit_message>
<xml_diff>
--- a/checkrates/week-18/Analisis_Checkrates_B2C_7d.xlsx
+++ b/checkrates/week-18/Analisis_Checkrates_B2C_7d.xlsx
@@ -541,7 +541,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 04:34 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 04:34 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 04:34 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 04:34 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -3734,7 +3734,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 04:34 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -5677,7 +5677,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 04:34 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -7489,18 +7489,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="41" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="25" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7520,7 +7520,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 04:34 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -7918,6 +7918,1406 @@
       <c r="I15" s="5" t="inlineStr">
         <is>
           <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Cartagena Area</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="n">
+        <v>4297</v>
+      </c>
+      <c r="D16" s="12" t="n">
+        <v>4139</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>35</v>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>0.9632301605771468</v>
+      </c>
+      <c r="G16" s="13" t="n">
+        <v>0.008145217593670002</v>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>Aceptable</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Revisar</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Atlanta Area</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="n">
+        <v>4295</v>
+      </c>
+      <c r="D17" s="12" t="n">
+        <v>4207</v>
+      </c>
+      <c r="E17" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" s="13" t="n">
+        <v>0.9795110593713621</v>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>0.0006984866123399302</v>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Mexico City - Central Mexico</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="n">
+        <v>3959</v>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>3807</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>160</v>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>0.9616064662793635</v>
+      </c>
+      <c r="G18" s="13" t="n">
+        <v>0.04041424602172266</v>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>Aceptable</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Seattle Area</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="n">
+        <v>3795</v>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>3612</v>
+      </c>
+      <c r="E19" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>0.9517786561264822</v>
+      </c>
+      <c r="G19" s="13" t="n">
+        <v>0.0007905138339920949</v>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>Aceptable</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Houston (and vicinity), TX, US</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="n">
+        <v>3341</v>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>3297</v>
+      </c>
+      <c r="E20" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>0.9868302903322359</v>
+      </c>
+      <c r="G20" s="13" t="n">
+        <v>0.002095181083507932</v>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Greenville Area</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>3281</v>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>2915</v>
+      </c>
+      <c r="E21" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="13" t="n">
+        <v>0.8884486437061871</v>
+      </c>
+      <c r="G21" s="13" t="n">
+        <v>0.0003047851264858275</v>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>Revisar</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="n">
+        <v>3071</v>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>2976</v>
+      </c>
+      <c r="E22" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>0.9690654509931619</v>
+      </c>
+      <c r="G22" s="13" t="n">
+        <v>0.001302507326603712</v>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>Aceptable</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Puerto Vallarta Area</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="n">
+        <v>3040</v>
+      </c>
+      <c r="D23" s="12" t="n">
+        <v>2962</v>
+      </c>
+      <c r="E23" s="12" t="n">
+        <v>35</v>
+      </c>
+      <c r="F23" s="13" t="n">
+        <v>0.9743421052631579</v>
+      </c>
+      <c r="G23" s="13" t="n">
+        <v>0.01151315789473684</v>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>Revisar</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Denver (and vicinity), CO, US</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="n">
+        <v>2950</v>
+      </c>
+      <c r="D24" s="12" t="n">
+        <v>2875</v>
+      </c>
+      <c r="E24" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>0.9745762711864406</v>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>0.0006779661016949153</v>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Nashville (and vicinity), TN, US</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="n">
+        <v>2893</v>
+      </c>
+      <c r="D25" s="12" t="n">
+        <v>2788</v>
+      </c>
+      <c r="E25" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" s="13" t="n">
+        <v>0.9637054960248876</v>
+      </c>
+      <c r="G25" s="13" t="n">
+        <v>0.001036985827860353</v>
+      </c>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>Aceptable</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Phoenix (and vicinity), AZ, US</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="n">
+        <v>2785</v>
+      </c>
+      <c r="D26" s="12" t="n">
+        <v>2731</v>
+      </c>
+      <c r="E26" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>0.9806104129263914</v>
+      </c>
+      <c r="G26" s="13" t="n">
+        <v>0.000718132854578097</v>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Acapulco</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>2758</v>
+      </c>
+      <c r="D27" s="12" t="n">
+        <v>2642</v>
+      </c>
+      <c r="E27" s="12" t="n">
+        <v>103</v>
+      </c>
+      <c r="F27" s="13" t="n">
+        <v>0.9579405366207396</v>
+      </c>
+      <c r="G27" s="13" t="n">
+        <v>0.03734590282813633</v>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>Aceptable</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Bogotá Area</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>2745</v>
+      </c>
+      <c r="D28" s="12" t="n">
+        <v>2347</v>
+      </c>
+      <c r="E28" s="12" t="n">
+        <v>55</v>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>0.8550091074681239</v>
+      </c>
+      <c r="G28" s="13" t="n">
+        <v>0.02003642987249545</v>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>Revisar</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Aceptable</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Honolulu Area</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>2660</v>
+      </c>
+      <c r="D29" s="12" t="n">
+        <v>2632</v>
+      </c>
+      <c r="E29" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" s="13" t="n">
+        <v>0.9894736842105263</v>
+      </c>
+      <c r="G29" s="13" t="n">
+        <v>0.0007518796992481203</v>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Montreal</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="n">
+        <v>2618</v>
+      </c>
+      <c r="D30" s="12" t="n">
+        <v>2590</v>
+      </c>
+      <c r="E30" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F30" s="13" t="n">
+        <v>0.9893048128342246</v>
+      </c>
+      <c r="G30" s="13" t="n">
+        <v>0.001145912910618793</v>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>New Orleans</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="n">
+        <v>2592</v>
+      </c>
+      <c r="D31" s="12" t="n">
+        <v>2558</v>
+      </c>
+      <c r="E31" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F31" s="13" t="n">
+        <v>0.9868827160493827</v>
+      </c>
+      <c r="G31" s="13" t="n">
+        <v>0.001157407407407407</v>
+      </c>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale (and vicinity), FL, US</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="n">
+        <v>2577</v>
+      </c>
+      <c r="D32" s="12" t="n">
+        <v>2551</v>
+      </c>
+      <c r="E32" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F32" s="13" t="n">
+        <v>0.9899107489328677</v>
+      </c>
+      <c r="G32" s="13" t="n">
+        <v>0.001552192471866511</v>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Niagara Falls, Canada</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="n">
+        <v>2525</v>
+      </c>
+      <c r="D33" s="12" t="n">
+        <v>2520</v>
+      </c>
+      <c r="E33" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="13" t="n">
+        <v>0.998019801980198</v>
+      </c>
+      <c r="G33" s="13" t="n">
+        <v>0.0003960396039603961</v>
+      </c>
+      <c r="H33" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Londres</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="n">
+        <v>2474</v>
+      </c>
+      <c r="D34" s="12" t="n">
+        <v>2332</v>
+      </c>
+      <c r="E34" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="13" t="n">
+        <v>0.9426030719482619</v>
+      </c>
+      <c r="G34" s="13" t="n">
+        <v>0.0004042037186742118</v>
+      </c>
+      <c r="H34" s="9" t="inlineStr">
+        <is>
+          <t>Aceptable</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Puerto Rico</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="n">
+        <v>2437</v>
+      </c>
+      <c r="D35" s="12" t="n">
+        <v>2415</v>
+      </c>
+      <c r="E35" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="13" t="n">
+        <v>0.9909725071809602</v>
+      </c>
+      <c r="G35" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>Sin Conversión</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Riviera Nayarit</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="n">
+        <v>2051</v>
+      </c>
+      <c r="D36" s="12" t="n">
+        <v>1507</v>
+      </c>
+      <c r="E36" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="F36" s="13" t="n">
+        <v>0.734763529985373</v>
+      </c>
+      <c r="G36" s="13" t="n">
+        <v>0.003412969283276451</v>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Punta Cana</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="n">
+        <v>2038</v>
+      </c>
+      <c r="D37" s="12" t="n">
+        <v>2019</v>
+      </c>
+      <c r="E37" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="F37" s="13" t="n">
+        <v>0.9906771344455348</v>
+      </c>
+      <c r="G37" s="13" t="n">
+        <v>0.01030421982335623</v>
+      </c>
+      <c r="H37" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>Revisar</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="n">
+        <v>1876</v>
+      </c>
+      <c r="D38" s="12" t="n">
+        <v>1852</v>
+      </c>
+      <c r="E38" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F38" s="13" t="n">
+        <v>0.9872068230277186</v>
+      </c>
+      <c r="G38" s="13" t="n">
+        <v>0.002132196162046908</v>
+      </c>
+      <c r="H38" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="n">
+        <v>1830</v>
+      </c>
+      <c r="D39" s="12" t="n">
+        <v>1789</v>
+      </c>
+      <c r="E39" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="13" t="n">
+        <v>0.9775956284153006</v>
+      </c>
+      <c r="G39" s="13" t="n">
+        <v>0.000546448087431694</v>
+      </c>
+      <c r="H39" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Philadelphia (and vicinity), PA, US</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="n">
+        <v>1711</v>
+      </c>
+      <c r="D40" s="12" t="n">
+        <v>1677</v>
+      </c>
+      <c r="E40" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="13" t="n">
+        <v>0.9801285797779077</v>
+      </c>
+      <c r="G40" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>Sin Conversión</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="n">
+        <v>1706</v>
+      </c>
+      <c r="D41" s="12" t="n">
+        <v>1643</v>
+      </c>
+      <c r="E41" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="F41" s="13" t="n">
+        <v>0.9630715123094959</v>
+      </c>
+      <c r="G41" s="13" t="n">
+        <v>0.007033997655334115</v>
+      </c>
+      <c r="H41" s="9" t="inlineStr">
+        <is>
+          <t>Aceptable</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Washington, DC Area</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="n">
+        <v>1534</v>
+      </c>
+      <c r="D42" s="12" t="n">
+        <v>1502</v>
+      </c>
+      <c r="E42" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" s="13" t="n">
+        <v>0.9791395045632334</v>
+      </c>
+      <c r="G42" s="13" t="n">
+        <v>0.001303780964797914</v>
+      </c>
+      <c r="H42" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Ixtapa / Zihuatanejo</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="n">
+        <v>1486</v>
+      </c>
+      <c r="D43" s="12" t="n">
+        <v>1365</v>
+      </c>
+      <c r="E43" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="F43" s="13" t="n">
+        <v>0.9185733512786003</v>
+      </c>
+      <c r="G43" s="13" t="n">
+        <v>0.008075370121130552</v>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>Revisar</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>Revisar</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Tampa Area</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="n">
+        <v>1465</v>
+      </c>
+      <c r="D44" s="12" t="n">
+        <v>1434</v>
+      </c>
+      <c r="E44" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="13" t="n">
+        <v>0.978839590443686</v>
+      </c>
+      <c r="G44" s="13" t="n">
+        <v>0.0006825938566552901</v>
+      </c>
+      <c r="H44" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Pittsburgh Area</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="n">
+        <v>1461</v>
+      </c>
+      <c r="D45" s="12" t="n">
+        <v>1446</v>
+      </c>
+      <c r="E45" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="13" t="n">
+        <v>0.9897330595482546</v>
+      </c>
+      <c r="G45" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>Sin Conversión</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Monterrey</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="n">
+        <v>1444</v>
+      </c>
+      <c r="D46" s="12" t="n">
+        <v>1143</v>
+      </c>
+      <c r="E46" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="F46" s="13" t="n">
+        <v>0.7915512465373962</v>
+      </c>
+      <c r="G46" s="13" t="n">
+        <v>0.04155124653739612</v>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Medellin Area</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="n">
+        <v>1426</v>
+      </c>
+      <c r="D47" s="12" t="n">
+        <v>1358</v>
+      </c>
+      <c r="E47" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="F47" s="13" t="n">
+        <v>0.9523141654978962</v>
+      </c>
+      <c r="G47" s="13" t="n">
+        <v>0.01332398316970547</v>
+      </c>
+      <c r="H47" s="9" t="inlineStr">
+        <is>
+          <t>Aceptable</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>Revisar</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Jacksonville Area</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="n">
+        <v>1321</v>
+      </c>
+      <c r="D48" s="12" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E48" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" s="13" t="n">
+        <v>0.9841029523088569</v>
+      </c>
+      <c r="G48" s="13" t="n">
+        <v>0.002271006813020439</v>
+      </c>
+      <c r="H48" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Aruba</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="n">
+        <v>1271</v>
+      </c>
+      <c r="D49" s="12" t="n">
+        <v>1237</v>
+      </c>
+      <c r="E49" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" s="13" t="n">
+        <v>0.973249409913454</v>
+      </c>
+      <c r="G49" s="13" t="n">
+        <v>0.002360346184107002</v>
+      </c>
+      <c r="H49" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Anaheim Area</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="n">
+        <v>1252</v>
+      </c>
+      <c r="D50" s="12" t="n">
+        <v>1236</v>
+      </c>
+      <c r="E50" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="F50" s="13" t="n">
+        <v>0.987220447284345</v>
+      </c>
+      <c r="G50" s="13" t="n">
+        <v>0.004792332268370607</v>
+      </c>
+      <c r="H50" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Minneapolis - St. Paul Area</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="n">
+        <v>1237</v>
+      </c>
+      <c r="D51" s="12" t="n">
+        <v>1214</v>
+      </c>
+      <c r="E51" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F51" s="13" t="n">
+        <v>0.9814066289409863</v>
+      </c>
+      <c r="G51" s="13" t="n">
+        <v>0.003233629749393694</v>
+      </c>
+      <c r="H51" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Detroit Area</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="n">
+        <v>1209</v>
+      </c>
+      <c r="D52" s="12" t="n">
+        <v>1192</v>
+      </c>
+      <c r="E52" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F52" s="13" t="n">
+        <v>0.9859387923904053</v>
+      </c>
+      <c r="G52" s="13" t="n">
+        <v>0.001654259718775848</v>
+      </c>
+      <c r="H52" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Santa Marta Area</t>
+        </is>
+      </c>
+      <c r="C53" s="12" t="n">
+        <v>1156</v>
+      </c>
+      <c r="D53" s="12" t="n">
+        <v>1145</v>
+      </c>
+      <c r="E53" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="F53" s="13" t="n">
+        <v>0.990484429065744</v>
+      </c>
+      <c r="G53" s="13" t="n">
+        <v>0.02076124567474048</v>
+      </c>
+      <c r="H53" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>Aceptable</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Mazatlán</t>
+        </is>
+      </c>
+      <c r="C54" s="12" t="n">
+        <v>1129</v>
+      </c>
+      <c r="D54" s="12" t="n">
+        <v>1119</v>
+      </c>
+      <c r="E54" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="F54" s="13" t="n">
+        <v>0.9911426040744021</v>
+      </c>
+      <c r="G54" s="13" t="n">
+        <v>0.01505757307351639</v>
+      </c>
+      <c r="H54" s="10" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>Aceptable</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>El Cairo Area</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="n">
+        <v>1128</v>
+      </c>
+      <c r="D55" s="12" t="n">
+        <v>1074</v>
+      </c>
+      <c r="E55" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="13" t="n">
+        <v>0.9521276595744681</v>
+      </c>
+      <c r="G55" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="9" t="inlineStr">
+        <is>
+          <t>Aceptable</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>Sin Conversión</t>
         </is>
       </c>
     </row>
@@ -7963,7 +9363,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 04:34 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>
@@ -8301,7 +9701,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 09/05/2026 04:34 · W18 · 27 abr – 3 may 2026</t>
+          <t>Generado: 09/05/2026 05:07 · W18 · 27 abr – 3 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>